<commit_message>
rawr v2 but use rawr :)
</commit_message>
<xml_diff>
--- a/leads_with_explanations.xlsx
+++ b/leads_with_explanations.xlsx
@@ -2,9 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
-  <workbookProtection/>
   <bookViews>
-    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
+    <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="240" yWindow="15" windowWidth="16095" windowHeight="9660" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
@@ -26,13 +25,16 @@
       <scheme val="minor"/>
     </font>
     <font>
+      <name val="Calibri"/>
+      <family val="2"/>
       <b val="1"/>
+      <color theme="1"/>
+      <sz val="11"/>
+      <scheme val="minor"/>
     </font>
     <font>
-      <name val="Arial"/>
       <b val="1"/>
       <color rgb="00FFFFFF"/>
-      <sz val="10"/>
     </font>
   </fonts>
   <fills count="3">
@@ -57,10 +59,19 @@
       <diagonal/>
     </border>
     <border>
-      <left style="thin"/>
-      <right style="thin"/>
-      <top style="thin"/>
-      <bottom style="thin"/>
+      <left style="thin">
+        <color auto="1"/>
+      </left>
+      <right style="thin">
+        <color auto="1"/>
+      </right>
+      <top style="thin">
+        <color auto="1"/>
+      </top>
+      <bottom style="thin">
+        <color auto="1"/>
+      </bottom>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -79,7 +90,7 @@
     </xf>
   </cellXfs>
   <cellStyles count="1">
-    <cellStyle name="Normal" xfId="0" builtinId="0" hidden="0"/>
+    <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium9" defaultPivotStyle="PivotStyleLight16"/>
   <colors>
@@ -442,130 +453,131 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:DN3"/>
+  <dimension ref="A1:DO3"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
-    <col width="18" customWidth="1" min="1" max="1"/>
-    <col width="18" customWidth="1" min="2" max="2"/>
-    <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="18" customWidth="1" min="4" max="4"/>
-    <col width="18" customWidth="1" min="5" max="5"/>
-    <col width="18" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="18" customWidth="1" min="8" max="8"/>
-    <col width="18" customWidth="1" min="9" max="9"/>
-    <col width="18" customWidth="1" min="10" max="10"/>
-    <col width="18" customWidth="1" min="11" max="11"/>
-    <col width="18" customWidth="1" min="12" max="12"/>
-    <col width="18" customWidth="1" min="13" max="13"/>
-    <col width="18" customWidth="1" min="14" max="14"/>
-    <col width="18" customWidth="1" min="15" max="15"/>
-    <col width="18" customWidth="1" min="16" max="16"/>
-    <col width="18" customWidth="1" min="17" max="17"/>
-    <col width="18" customWidth="1" min="18" max="18"/>
-    <col width="18" customWidth="1" min="19" max="19"/>
-    <col width="18" customWidth="1" min="20" max="20"/>
-    <col width="18" customWidth="1" min="21" max="21"/>
-    <col width="18" customWidth="1" min="22" max="22"/>
-    <col width="18" customWidth="1" min="23" max="23"/>
-    <col width="18" customWidth="1" min="24" max="24"/>
-    <col width="18" customWidth="1" min="25" max="25"/>
-    <col width="18" customWidth="1" min="26" max="26"/>
-    <col width="18" customWidth="1" min="27" max="27"/>
-    <col width="18" customWidth="1" min="28" max="28"/>
-    <col width="18" customWidth="1" min="29" max="29"/>
-    <col width="18" customWidth="1" min="30" max="30"/>
-    <col width="18" customWidth="1" min="31" max="31"/>
-    <col width="18" customWidth="1" min="32" max="32"/>
-    <col width="18" customWidth="1" min="33" max="33"/>
-    <col width="18" customWidth="1" min="34" max="34"/>
-    <col width="18" customWidth="1" min="35" max="35"/>
-    <col width="18" customWidth="1" min="36" max="36"/>
-    <col width="18" customWidth="1" min="37" max="37"/>
-    <col width="18" customWidth="1" min="38" max="38"/>
-    <col width="18" customWidth="1" min="39" max="39"/>
-    <col width="18" customWidth="1" min="40" max="40"/>
-    <col width="18" customWidth="1" min="41" max="41"/>
-    <col width="18" customWidth="1" min="42" max="42"/>
-    <col width="18" customWidth="1" min="43" max="43"/>
-    <col width="18" customWidth="1" min="44" max="44"/>
-    <col width="18" customWidth="1" min="45" max="45"/>
-    <col width="18" customWidth="1" min="46" max="46"/>
-    <col width="18" customWidth="1" min="47" max="47"/>
-    <col width="18" customWidth="1" min="48" max="48"/>
-    <col width="18" customWidth="1" min="49" max="49"/>
-    <col width="18" customWidth="1" min="50" max="50"/>
-    <col width="18" customWidth="1" min="51" max="51"/>
-    <col width="18" customWidth="1" min="52" max="52"/>
-    <col width="18" customWidth="1" min="53" max="53"/>
-    <col width="18" customWidth="1" min="54" max="54"/>
-    <col width="18" customWidth="1" min="55" max="55"/>
-    <col width="18" customWidth="1" min="56" max="56"/>
-    <col width="18" customWidth="1" min="57" max="57"/>
-    <col width="18" customWidth="1" min="58" max="58"/>
-    <col width="18" customWidth="1" min="59" max="59"/>
-    <col width="18" customWidth="1" min="60" max="60"/>
-    <col width="18" customWidth="1" min="61" max="61"/>
-    <col width="18" customWidth="1" min="62" max="62"/>
-    <col width="18" customWidth="1" min="63" max="63"/>
-    <col width="18" customWidth="1" min="64" max="64"/>
-    <col width="18" customWidth="1" min="65" max="65"/>
-    <col width="18" customWidth="1" min="66" max="66"/>
-    <col width="18" customWidth="1" min="67" max="67"/>
-    <col width="18" customWidth="1" min="68" max="68"/>
-    <col width="18" customWidth="1" min="69" max="69"/>
-    <col width="18" customWidth="1" min="70" max="70"/>
-    <col width="18" customWidth="1" min="71" max="71"/>
-    <col width="18" customWidth="1" min="72" max="72"/>
-    <col width="18" customWidth="1" min="73" max="73"/>
-    <col width="18" customWidth="1" min="74" max="74"/>
-    <col width="18" customWidth="1" min="75" max="75"/>
-    <col width="18" customWidth="1" min="76" max="76"/>
-    <col width="18" customWidth="1" min="77" max="77"/>
-    <col width="18" customWidth="1" min="78" max="78"/>
-    <col width="18" customWidth="1" min="79" max="79"/>
-    <col width="18" customWidth="1" min="80" max="80"/>
-    <col width="18" customWidth="1" min="81" max="81"/>
-    <col width="18" customWidth="1" min="82" max="82"/>
-    <col width="18" customWidth="1" min="83" max="83"/>
-    <col width="18" customWidth="1" min="84" max="84"/>
-    <col width="18" customWidth="1" min="85" max="85"/>
-    <col width="18" customWidth="1" min="86" max="86"/>
-    <col width="18" customWidth="1" min="87" max="87"/>
-    <col width="18" customWidth="1" min="88" max="88"/>
-    <col width="18" customWidth="1" min="89" max="89"/>
-    <col width="18" customWidth="1" min="90" max="90"/>
-    <col width="18" customWidth="1" min="91" max="91"/>
-    <col width="18" customWidth="1" min="92" max="92"/>
-    <col width="18" customWidth="1" min="93" max="93"/>
-    <col width="18" customWidth="1" min="94" max="94"/>
-    <col width="18" customWidth="1" min="95" max="95"/>
-    <col width="18" customWidth="1" min="96" max="96"/>
-    <col width="18" customWidth="1" min="97" max="97"/>
-    <col width="18" customWidth="1" min="98" max="98"/>
-    <col width="18" customWidth="1" min="99" max="99"/>
-    <col width="18" customWidth="1" min="100" max="100"/>
-    <col width="18" customWidth="1" min="101" max="101"/>
-    <col width="18" customWidth="1" min="102" max="102"/>
-    <col width="18" customWidth="1" min="103" max="103"/>
-    <col width="18" customWidth="1" min="104" max="104"/>
-    <col width="18" customWidth="1" min="105" max="105"/>
-    <col width="18" customWidth="1" min="106" max="106"/>
-    <col width="18" customWidth="1" min="107" max="107"/>
-    <col width="18" customWidth="1" min="108" max="108"/>
-    <col width="18" customWidth="1" min="109" max="109"/>
-    <col width="18" customWidth="1" min="110" max="110"/>
-    <col width="18" customWidth="1" min="111" max="111"/>
-    <col width="18" customWidth="1" min="112" max="112"/>
-    <col width="18" customWidth="1" min="113" max="113"/>
-    <col width="18" customWidth="1" min="114" max="114"/>
-    <col width="18" customWidth="1" min="115" max="115"/>
+    <col width="20" customWidth="1" min="1" max="1"/>
+    <col width="20" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="20" customWidth="1" min="4" max="4"/>
+    <col width="20" customWidth="1" min="5" max="5"/>
+    <col width="20" customWidth="1" min="6" max="6"/>
+    <col width="20" customWidth="1" min="7" max="7"/>
+    <col width="20" customWidth="1" min="8" max="8"/>
+    <col width="20" customWidth="1" min="9" max="9"/>
+    <col width="20" customWidth="1" min="10" max="10"/>
+    <col width="20" customWidth="1" min="11" max="11"/>
+    <col width="20" customWidth="1" min="12" max="12"/>
+    <col width="20" customWidth="1" min="13" max="13"/>
+    <col width="20" customWidth="1" min="14" max="14"/>
+    <col width="20" customWidth="1" min="15" max="15"/>
+    <col width="20" customWidth="1" min="16" max="16"/>
+    <col width="20" customWidth="1" min="17" max="17"/>
+    <col width="20" customWidth="1" min="18" max="18"/>
+    <col width="20" customWidth="1" min="19" max="19"/>
+    <col width="20" customWidth="1" min="20" max="20"/>
+    <col width="20" customWidth="1" min="21" max="21"/>
+    <col width="20" customWidth="1" min="22" max="22"/>
+    <col width="20" customWidth="1" min="23" max="23"/>
+    <col width="20" customWidth="1" min="24" max="24"/>
+    <col width="20" customWidth="1" min="25" max="25"/>
+    <col width="20" customWidth="1" min="26" max="26"/>
+    <col width="20" customWidth="1" min="27" max="27"/>
+    <col width="20" customWidth="1" min="28" max="28"/>
+    <col width="20" customWidth="1" min="29" max="29"/>
+    <col width="20" customWidth="1" min="30" max="30"/>
+    <col width="20" customWidth="1" min="31" max="31"/>
+    <col width="20" customWidth="1" min="32" max="32"/>
+    <col width="20" customWidth="1" min="33" max="33"/>
+    <col width="20" customWidth="1" min="34" max="34"/>
+    <col width="20" customWidth="1" min="35" max="35"/>
+    <col width="20" customWidth="1" min="36" max="36"/>
+    <col width="20" customWidth="1" min="37" max="37"/>
+    <col width="20" customWidth="1" min="38" max="38"/>
+    <col width="20" customWidth="1" min="39" max="39"/>
+    <col width="20" customWidth="1" min="40" max="40"/>
+    <col width="20" customWidth="1" min="41" max="41"/>
+    <col width="20" customWidth="1" min="42" max="42"/>
+    <col width="20" customWidth="1" min="43" max="43"/>
+    <col width="20" customWidth="1" min="44" max="44"/>
+    <col width="20" customWidth="1" min="45" max="45"/>
+    <col width="20" customWidth="1" min="46" max="46"/>
+    <col width="20" customWidth="1" min="47" max="47"/>
+    <col width="20" customWidth="1" min="48" max="48"/>
+    <col width="20" customWidth="1" min="49" max="49"/>
+    <col width="20" customWidth="1" min="50" max="50"/>
+    <col width="20" customWidth="1" min="51" max="51"/>
+    <col width="20" customWidth="1" min="52" max="52"/>
+    <col width="20" customWidth="1" min="53" max="53"/>
+    <col width="20" customWidth="1" min="54" max="54"/>
+    <col width="20" customWidth="1" min="55" max="55"/>
+    <col width="20" customWidth="1" min="56" max="56"/>
+    <col width="20" customWidth="1" min="57" max="57"/>
+    <col width="20" customWidth="1" min="58" max="58"/>
+    <col width="20" customWidth="1" min="59" max="59"/>
+    <col width="20" customWidth="1" min="60" max="60"/>
+    <col width="20" customWidth="1" min="61" max="61"/>
+    <col width="20" customWidth="1" min="62" max="62"/>
+    <col width="20" customWidth="1" min="63" max="63"/>
+    <col width="20" customWidth="1" min="64" max="64"/>
+    <col width="20" customWidth="1" min="65" max="65"/>
+    <col width="20" customWidth="1" min="66" max="66"/>
+    <col width="20" customWidth="1" min="67" max="67"/>
+    <col width="20" customWidth="1" min="68" max="68"/>
+    <col width="20" customWidth="1" min="69" max="69"/>
+    <col width="20" customWidth="1" min="70" max="70"/>
+    <col width="20" customWidth="1" min="71" max="71"/>
+    <col width="20" customWidth="1" min="72" max="72"/>
+    <col width="20" customWidth="1" min="73" max="73"/>
+    <col width="20" customWidth="1" min="74" max="74"/>
+    <col width="20" customWidth="1" min="75" max="75"/>
+    <col width="20" customWidth="1" min="76" max="76"/>
+    <col width="20" customWidth="1" min="77" max="77"/>
+    <col width="20" customWidth="1" min="78" max="78"/>
+    <col width="20" customWidth="1" min="79" max="79"/>
+    <col width="20" customWidth="1" min="80" max="80"/>
+    <col width="20" customWidth="1" min="81" max="81"/>
+    <col width="20" customWidth="1" min="82" max="82"/>
+    <col width="20" customWidth="1" min="83" max="83"/>
+    <col width="20" customWidth="1" min="84" max="84"/>
+    <col width="20" customWidth="1" min="85" max="85"/>
+    <col width="20" customWidth="1" min="86" max="86"/>
+    <col width="20" customWidth="1" min="87" max="87"/>
+    <col width="20" customWidth="1" min="88" max="88"/>
+    <col width="20" customWidth="1" min="89" max="89"/>
+    <col width="20" customWidth="1" min="90" max="90"/>
+    <col width="20" customWidth="1" min="91" max="91"/>
+    <col width="20" customWidth="1" min="92" max="92"/>
+    <col width="20" customWidth="1" min="93" max="93"/>
+    <col width="20" customWidth="1" min="94" max="94"/>
+    <col width="20" customWidth="1" min="95" max="95"/>
+    <col width="20" customWidth="1" min="96" max="96"/>
+    <col width="20" customWidth="1" min="97" max="97"/>
+    <col width="20" customWidth="1" min="98" max="98"/>
+    <col width="20" customWidth="1" min="99" max="99"/>
+    <col width="20" customWidth="1" min="100" max="100"/>
+    <col width="20" customWidth="1" min="101" max="101"/>
+    <col width="20" customWidth="1" min="102" max="102"/>
+    <col width="20" customWidth="1" min="103" max="103"/>
+    <col width="20" customWidth="1" min="104" max="104"/>
+    <col width="20" customWidth="1" min="105" max="105"/>
+    <col width="20" customWidth="1" min="106" max="106"/>
+    <col width="20" customWidth="1" min="107" max="107"/>
+    <col width="20" customWidth="1" min="108" max="108"/>
+    <col width="20" customWidth="1" min="109" max="109"/>
+    <col width="20" customWidth="1" min="110" max="110"/>
+    <col width="20" customWidth="1" min="111" max="111"/>
+    <col width="20" customWidth="1" min="112" max="112"/>
+    <col width="20" customWidth="1" min="113" max="113"/>
+    <col width="20" customWidth="1" min="114" max="114"/>
+    <col width="20" customWidth="1" min="115" max="115"/>
     <col width="80" customWidth="1" min="116" max="116"/>
     <col width="60" customWidth="1" min="117" max="117"/>
-    <col width="18" customWidth="1" min="118" max="118"/>
+    <col width="20" customWidth="1" min="118" max="118"/>
+    <col width="20" customWidth="1" min="119" max="119"/>
   </cols>
   <sheetData>
-    <row r="1" ht="30" customHeight="1">
+    <row r="1">
       <c r="A1" s="2" t="inlineStr">
         <is>
           <t>Lead_ID</t>
@@ -1154,6 +1166,11 @@
       <c r="DN1" s="2" t="inlineStr">
         <is>
           <t>llm_duration_sec</t>
+        </is>
+      </c>
+      <c r="DO1" s="2" t="inlineStr">
+        <is>
+          <t>validation_passed</t>
         </is>
       </c>
     </row>
@@ -1603,62 +1620,99 @@
       </c>
       <c r="DL2" s="3" t="inlineStr">
         <is>
-          <t>Here's a storytelling paragraph that explains the lead to a sales representative:
-We have a converted lead from LinkedIn, Avflight Corporation, with a predicted conversion probability of 4.6%. This COLD-rated lead has shown strong engagement signals, including high ad impressions and time on site, indicating a genuine interest in our Safety Systems product for their Bombardier Global 7500 aircraft. The fact that they have a corporate email address and are aware of the source (LinkedIn) suggests a level of professionalism and intent to purchase. However, there are some concerns - their loyalty score is low, and existing customer validity is not aligned with the lead's profile. To move forward, I recommend reaching out via email to discuss their specific needs and pain points, leveraging the positive signals from their engagement history.</t>
+          <t>Based on the provided evidence, lead LD-100015 from Avflight Corporation has a predicted conversion likelihood of 4.64%. The strongest positive drivers contributing to this likelihood are Ad Impressions, Time on Site, Purchase History, Engagement Rate, and Email Opens. Conversely, Trial Conversions, Referral Source, Location Score, Device Type, and Plan Type are the strongest negative drivers reducing qualification likelihood. Given these factors, I recommend conducting additional qualification before prioritizing sales outreach.</t>
         </is>
       </c>
       <c r="DM2" t="inlineStr">
         <is>
-          <t>Based on the following lead data, write a storytelling paragraph that explains this lead 
-to a sales representative in a natural, insightful, and action-oriented way.
-LEAD SUMMARY
-------------
-Lead ID       : LD-100015
-Company       : Avflight Corporation
-Lead Status   : Converted
-Lead Source   : LinkedIn
-Region        : EMEA / Western Europe
-Market        : Commercial Aviation
-Account Type  : Partner
-Product       : Safety Systems
-Aircraft      : Bombardier Global 7500
-Est. Value    : $4,209,443
-Loyalty       : Low
-Account Exists: Yes
-Phone         : Not Available
-Corporate Email: Yes
-MODEL SCORES
-------------
-Predicted Conversion Probability : 4.6%
-Lead Rating                      : COLD
-AQL Category                     : Aql Accept
-Behavior Score                   : 34.8/100
-Demographic Score                : 51.4/100
-Engagement Score                 : 70.5/100
-Confidence                       : 90.7%
-KEY CONVERSION DRIVERS (from SHAP analysis)
---------------------------------------------
-Positive Signals:
-  (+) Ad Impressions: strongly supports conversion
-  (+) Time on Site: strongly supports conversion
-  (+) Purchase History: strongly supports conversion
-  (+) Engagement Rate: strongly supports conversion
-  (+) Email Opens: strongly supports conversion
-Negative Signals:
-  (-) Trial Conversions: acts as a barrier to conversion
-  (-) Referral Source: acts as a barrier to conversion
-  (-) Location Score: acts as a barrier to conversion
-  (-) Device Type: acts as a barrier to conversion
-  (-) Plan Type: acts as a barrier to conversion
-TOPIC ALIGNMENT SIGNALS
------------------------
-Aligned    : Lead Description Completeness, Lead Score &amp; Stage, Corporate Email Address, Source Awareness, Strong Commercial Intent, FSE Generated Lead
-Not Aligned: Existing Customer Validity, Early Intent Signal
-Your narrative paragraph:</t>
+          <t>Generate a factual lead explanation using ONLY the evidence below.
+EVIDENCE:
+{
+  "lead_summary": {
+    "lead_id": "LD-100015",
+    "company": "Avflight Corporation",
+    "lead_rating": "Cold",
+    "predicted_probability": 0.0464,
+    "confidence_level": "shows limited evidence of",
+    "product_interest": "Safety Systems",
+    "market": "Commercial Aviation"
+  },
+  "positive_evidence": [
+    {
+      "feature": "Ad Impressions",
+      "shap": 1.4401,
+      "meaning": "Ad Impressions contributed positively to qualification likelihood."
+    },
+    {
+      "feature": "Time on Site",
+      "shap": 1.3486,
+      "meaning": "Time on Site contributed positively to qualification likelihood."
+    },
+    {
+      "feature": "Purchase History",
+      "shap": 1.2798,
+      "meaning": "Purchase History contributed positively to qualification likelihood."
+    },
+    {
+      "feature": "Engagement Rate",
+      "shap": 1.1904,
+      "meaning": "Engagement Rate contributed positively to qualification likelihood."
+    },
+    {
+      "feature": "Email Opens",
+      "shap": 1.0871,
+      "meaning": "Email Opens contributed positively to qualification likelihood."
+    }
+  ],
+  "negative_evidence": [
+    {
+      "feature": "Trial Conversions",
+      "shap": -1.3774,
+      "meaning": "Trial Conversions reduced qualification likelihood."
+    },
+    {
+      "feature": "Referral Source",
+      "shap": -1.2724,
+      "meaning": "Referral Source reduced qualification likelihood."
+    },
+    {
+      "feature": "Location Score",
+      "shap": -1.1159,
+      "meaning": "Location Score reduced qualification likelihood."
+    },
+    {
+      "feature": "Device Type",
+      "shap": -1.1134,
+      "meaning": "Device Type reduced qualification likelihood."
+    },
+    {
+      "feature": "Plan Type",
+      "shap": -1.0835,
+      "meaning": "Plan Type reduced qualification likelihood."
+    }
+  ],
+  "aligned_topics": [
+    "Lead Description Completeness",
+    "Lead Score &amp; Stage",
+    "Corporate Email Address",
+    "Source Awareness",
+    "Strong Commercial Intent",
+    "FSE Generated Lead"
+  ],
+  "not_aligned_topics": [
+    "Existing Customer Validity",
+    "Early Intent Signal"
+  ],
+  "recommended_action": "Conduct additional qualification before prioritizing sales outreach."
+}
+Write one concise business paragraph.</t>
         </is>
       </c>
       <c r="DN2" t="n">
-        <v>87.23</v>
+        <v>121.93</v>
+      </c>
+      <c r="DO2" t="b">
+        <v>1</v>
       </c>
     </row>
     <row r="3">
@@ -2107,65 +2161,102 @@
       </c>
       <c r="DL3" s="3" t="inlineStr">
         <is>
-          <t>Here is the narrative paragraph:
-As you review this lead, LD-100017 from Wheels Up Partners, a competitor in the MRO market, we see some promising signs. The estimated value of $741,743 for an Avionics Upgrade on their Bombardier Global 7500 aircraft suggests a significant potential sale. While the predicted conversion probability is lower at 26.9%, the lead's behavior score of 89.1/100 indicates strong engagement with our content. However, we also see some red flags, including low email open rates and a location score that may impact conversion. Notably, cart abandonment, trial conversions, revenue potential, lead behavior, and purchase history all strongly support conversion. To move this lead forward, I recommend reaching out via corporate email to gauge their interest in our solution and address any concerns they may have about the demo request process. By doing so, we can overcome some of the negative signals and capitalize on the positive ones to drive a successful sale.</t>
+          <t>Based on the provided evidence, lead LD-100017 from Wheels Up Partners has a predicted conversion likelihood of 26.88%. The strongest positive drivers contributing to this likelihood include Cart Abandonment, Trial Conversions, Revenue Potential, Lead Behavior, and Purchase History. Conversely, Demo Requests, Email Opens, Location Score, API Calls, and Session Duration are the strongest negative drivers reducing qualification likelihood. Given these factors, I recommend conducting additional qualification before prioritizing sales outreach.</t>
         </is>
       </c>
       <c r="DM3" t="inlineStr">
         <is>
-          <t>Based on the following lead data, write a storytelling paragraph that explains this lead 
-to a sales representative in a natural, insightful, and action-oriented way.
-LEAD SUMMARY
-------------
-Lead ID       : LD-100017
-Company       : Wheels Up Partners
-Lead Status   : Unqualified
-Lead Source   : Cold Call
-Region        : Asia Pacific / West Coast US
-Market        : MRO
-Account Type  : Competitor
-Product       : Avionics Upgrade
-Aircraft      : Bombardier Global 7500
-Est. Value    : $741,743
-Loyalty       : Medium
-Account Exists: No
-Phone         : Not Available
-Corporate Email: Yes
-MODEL SCORES
-------------
-Predicted Conversion Probability : 26.9%
-Lead Rating                      : COLD
-AQL Category                     : Disqualify Nurture
-Behavior Score                   : 89.1/100
-Demographic Score                : 59.4/100
-Engagement Score                 : 61.1/100
-Confidence                       : 46.2%
-KEY CONVERSION DRIVERS (from SHAP analysis)
---------------------------------------------
-Positive Signals:
-  (+) Cart Abandonment: strongly supports conversion
-  (+) Trial Conversions: strongly supports conversion
-  (+) Revenue Potential: strongly supports conversion
-  (+) Lead Behavior: strongly supports conversion
-  (+) Purchase History: strongly supports conversion
-Negative Signals:
-  (-) Demo Requests: acts as a barrier to conversion
-  (-) Email Opens: acts as a barrier to conversion
-  (-) Location Score: acts as a barrier to conversion
-  (-) API Calls: acts as a barrier to conversion
-  (-) Session Duration: acts as a barrier to conversion
-TOPIC ALIGNMENT SIGNALS
------------------------
-Aligned    : Corporate Email Address, Existing Customer Validity, Source Awareness, Early Intent Signal, Strong Commercial Intent
-Not Aligned: Lead Description Completeness, Lead Score &amp; Stage, FSE Generated Lead
-Your narrative paragraph:</t>
+          <t>Generate a factual lead explanation using ONLY the evidence below.
+EVIDENCE:
+{
+  "lead_summary": {
+    "lead_id": "LD-100017",
+    "company": "Wheels Up Partners",
+    "lead_rating": "Cold",
+    "predicted_probability": 0.2688,
+    "confidence_level": "shows limited evidence of",
+    "product_interest": "Avionics Upgrade",
+    "market": "MRO"
+  },
+  "positive_evidence": [
+    {
+      "feature": "Cart Abandonment",
+      "shap": 1.4595,
+      "meaning": "Cart Abandonment contributed positively to qualification likelihood."
+    },
+    {
+      "feature": "Trial Conversions",
+      "shap": 1.4471,
+      "meaning": "Trial Conversions contributed positively to qualification likelihood."
+    },
+    {
+      "feature": "Revenue Potential",
+      "shap": 1.1903,
+      "meaning": "Revenue Potential contributed positively to qualification likelihood."
+    },
+    {
+      "feature": "Lead Behavior",
+      "shap": 0.8675,
+      "meaning": "Lead Behavior contributed positively to qualification likelihood."
+    },
+    {
+      "feature": "Purchase History",
+      "shap": 0.7363,
+      "meaning": "Purchase History contributed positively to qualification likelihood."
+    }
+  ],
+  "negative_evidence": [
+    {
+      "feature": "Demo Requests",
+      "shap": -1.2593,
+      "meaning": "Demo Requests reduced qualification likelihood."
+    },
+    {
+      "feature": "Email Opens",
+      "shap": -1.2392,
+      "meaning": "Email Opens reduced qualification likelihood."
+    },
+    {
+      "feature": "Location Score",
+      "shap": -1.1947,
+      "meaning": "Location Score reduced qualification likelihood."
+    },
+    {
+      "feature": "API Calls",
+      "shap": -1.1639,
+      "meaning": "API Calls reduced qualification likelihood."
+    },
+    {
+      "feature": "Session Duration",
+      "shap": -1.1173,
+      "meaning": "Session Duration reduced qualification likelihood."
+    }
+  ],
+  "aligned_topics": [
+    "Corporate Email Address",
+    "Existing Customer Validity",
+    "Source Awareness",
+    "Early Intent Signal",
+    "Strong Commercial Intent"
+  ],
+  "not_aligned_topics": [
+    "Lead Description Completeness",
+    "Lead Score &amp; Stage",
+    "FSE Generated Lead"
+  ],
+  "recommended_action": "Conduct additional qualification before prioritizing sales outreach."
+}
+Write one concise business paragraph.</t>
         </is>
       </c>
       <c r="DN3" t="n">
-        <v>93.51000000000001</v>
+        <v>108.68</v>
+      </c>
+      <c r="DO3" t="b">
+        <v>1</v>
       </c>
     </row>
   </sheetData>
-  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
</xml_diff>